<commit_message>
update to measure reaction times of critical items
</commit_message>
<xml_diff>
--- a/resources/stimuliMainTask.xlsx
+++ b/resources/stimuliMainTask.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\medej\Desktop\scalar-implicatures\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marie\Desktop\Experiment Semantiek Pragmatiek\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{381EF701-FE27-43BF-A2F9-2834D22541A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D05B63EB-B33B-41BC-8BC4-CF69D3B796D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$45</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="193">
   <si>
     <t>condition</t>
   </si>
@@ -114,9 +114,6 @@
     <t>test</t>
   </si>
   <si>
-    <t>sentence</t>
-  </si>
-  <si>
     <t>id</t>
   </si>
   <si>
@@ -135,30 +132,9 @@
     <t>Paul</t>
   </si>
   <si>
-    <t>l'actrice n'est pas sublime</t>
-  </si>
-  <si>
-    <t>negation</t>
-  </si>
-  <si>
-    <t>le train est rapide</t>
-  </si>
-  <si>
-    <t>l’actrice est belle</t>
-  </si>
-  <si>
-    <t>le train n'est pas lent</t>
-  </si>
-  <si>
     <t>Julie</t>
   </si>
   <si>
-    <t>la peinture est large</t>
-  </si>
-  <si>
-    <t>la peinture n'est pas colorée</t>
-  </si>
-  <si>
     <t>noir/blanc</t>
   </si>
   <si>
@@ -186,286 +162,451 @@
     <t>large/colorée</t>
   </si>
   <si>
-    <t>la cuisine est sale</t>
-  </si>
-  <si>
-    <t>la cuisine n'est pas propre</t>
-  </si>
-  <si>
-    <t>l'homme est pauvre</t>
-  </si>
-  <si>
-    <t>l'homme n'est pas riche</t>
-  </si>
-  <si>
-    <t>l'histoire est superficielle</t>
-  </si>
-  <si>
-    <t>l'histoire n'est pas profonde</t>
-  </si>
-  <si>
-    <t>le bébé est petit</t>
-  </si>
-  <si>
-    <t>le bébé n'est pas grand</t>
-  </si>
-  <si>
-    <t>le chien est gentil</t>
-  </si>
-  <si>
-    <t>le chien n'est pas méchant</t>
-  </si>
-  <si>
-    <t>le magasin est fermé</t>
-  </si>
-  <si>
-    <t>le magasin n'est pas ouvert</t>
-  </si>
-  <si>
-    <t>le garçon est actif</t>
-  </si>
-  <si>
-    <t>le garçon n'est pas paresseux</t>
-  </si>
-  <si>
     <t>froid/chaud</t>
   </si>
   <si>
-    <t>le thé est froid</t>
-  </si>
-  <si>
-    <t>le thé n'est pas chaud</t>
-  </si>
-  <si>
-    <t>le collier est spéciale</t>
-  </si>
-  <si>
-    <t>le collier n'est pas unique</t>
-  </si>
-  <si>
-    <t>la pile est faible</t>
-  </si>
-  <si>
-    <t>la pile n'est pas vide</t>
-  </si>
-  <si>
-    <t>la tâche est dure</t>
-  </si>
-  <si>
-    <t>la tache n'est pas insoluble</t>
-  </si>
-  <si>
-    <t>le voyage est mémorable</t>
-  </si>
-  <si>
-    <t>le voyage n'est pas inoubliable</t>
-  </si>
-  <si>
-    <t>l'athlète est fatigué</t>
-  </si>
-  <si>
-    <t>l'athlète n'est pas épuisé</t>
-  </si>
-  <si>
-    <t>la classe est calme</t>
-  </si>
-  <si>
-    <t>la classe n'est pas inaudible</t>
-  </si>
-  <si>
-    <t>la serviette est mouillée</t>
-  </si>
-  <si>
-    <t>la serviette n'est pas trempée</t>
-  </si>
-  <si>
-    <t>la fille est triste</t>
-  </si>
-  <si>
-    <t>la fille n'est pas abattue</t>
-  </si>
-  <si>
-    <t>le test est difficile</t>
-  </si>
-  <si>
-    <t>le test n'est pas impossible</t>
-  </si>
-  <si>
-    <t>la réponse est bonne</t>
-  </si>
-  <si>
-    <t>la réponse n'est pas parfaite</t>
-  </si>
-  <si>
-    <t>le soldat est respectable</t>
-  </si>
-  <si>
-    <t>le soldat n'est pas honorable</t>
-  </si>
-  <si>
-    <t>la lumière est vive</t>
-  </si>
-  <si>
-    <t>la lumière n'est pas éblouissante</t>
-  </si>
-  <si>
-    <t>le repas est goûteux</t>
-  </si>
-  <si>
-    <t>le repas n'est pas délicieux</t>
-  </si>
-  <si>
-    <t>la statue est vieille</t>
-  </si>
-  <si>
-    <t>la statue n'est pas ancienne</t>
-  </si>
-  <si>
-    <t>le bâtiment est gros</t>
-  </si>
-  <si>
-    <t>le bâtiment n'est pas énorme</t>
-  </si>
-  <si>
-    <t>le cuisinier est gras</t>
-  </si>
-  <si>
-    <t>le cuisinier n'est pas obèse</t>
-  </si>
-  <si>
-    <t>le voyageur a faim</t>
-  </si>
-  <si>
-    <t>le voyageur n'est pas affamé</t>
-  </si>
-  <si>
-    <t>le cheval est noir</t>
-  </si>
-  <si>
-    <t>le cheval n'est pas blanc</t>
-  </si>
-  <si>
-    <t>le chat est mignon</t>
-  </si>
-  <si>
-    <t>le chat n'est pas beau</t>
-  </si>
-  <si>
-    <t>la blague est drôle</t>
-  </si>
-  <si>
-    <t>la blague n'est pas hilarante</t>
-  </si>
-  <si>
-    <t>le portrait est moche</t>
-  </si>
-  <si>
-    <t>le chercheur est intelligent</t>
-  </si>
-  <si>
-    <t>le chercheur n'est pas briljant</t>
-  </si>
-  <si>
-    <t>le portrait n'est pas hideux</t>
-  </si>
-  <si>
     <t>léger/lourd</t>
   </si>
   <si>
-    <t>le sac est léger</t>
-  </si>
-  <si>
-    <t>le sac n'est pas lourd</t>
-  </si>
-  <si>
-    <t>le modèle est joli</t>
-  </si>
-  <si>
     <t>joli/fort</t>
   </si>
   <si>
-    <t>le modèle n'est pas fort</t>
-  </si>
-  <si>
-    <t>l'enfant est timide</t>
-  </si>
-  <si>
     <t>timide/curieux</t>
   </si>
   <si>
-    <t>l'enfant n'est pas curieux</t>
-  </si>
-  <si>
     <t>fou/dangereux</t>
   </si>
   <si>
-    <t>le criminel est fou</t>
-  </si>
-  <si>
-    <t>le clown n'est pas dangereux</t>
-  </si>
-  <si>
-    <t>l'ours est effrayant</t>
-  </si>
-  <si>
     <t>effrayant/marron</t>
   </si>
   <si>
-    <t>l'ours n'est pas marron</t>
-  </si>
-  <si>
-    <t>le professeur est fâché</t>
-  </si>
-  <si>
     <t>fâché/raisonnable</t>
   </si>
   <si>
-    <t>le professeur n'est pas strict</t>
-  </si>
-  <si>
-    <t>la robe est chère</t>
-  </si>
-  <si>
     <t>cher/ennuyeuse</t>
   </si>
   <si>
-    <t>la robe n'est pas ennuyeuse</t>
-  </si>
-  <si>
-    <t>la couverture est douce</t>
-  </si>
-  <si>
-    <t>la couverture n'est pas fine</t>
-  </si>
-  <si>
     <t>doux/fin</t>
   </si>
   <si>
-    <t>l'étudiant est jeune</t>
-  </si>
-  <si>
     <t>jeune/sérieux</t>
   </si>
   <si>
-    <t>l'étudiant n'est pas sérieux</t>
-  </si>
-  <si>
-    <t>le propriétaire est poli</t>
-  </si>
-  <si>
-    <t>le propriétaire n'est pas pressé</t>
-  </si>
-  <si>
     <t>poli/pressé</t>
   </si>
   <si>
-    <t>le candidat est stupide</t>
-  </si>
-  <si>
-    <t>le candidat n'est pas inquiet</t>
-  </si>
-  <si>
     <t>stupide/inquiet</t>
+  </si>
+  <si>
+    <t>subject</t>
+  </si>
+  <si>
+    <t>le collier</t>
+  </si>
+  <si>
+    <t>la pile</t>
+  </si>
+  <si>
+    <t>la tâche</t>
+  </si>
+  <si>
+    <t>le voyage</t>
+  </si>
+  <si>
+    <t>la classe</t>
+  </si>
+  <si>
+    <t>la serviette</t>
+  </si>
+  <si>
+    <t>la fille</t>
+  </si>
+  <si>
+    <t>le test</t>
+  </si>
+  <si>
+    <t>la réponse</t>
+  </si>
+  <si>
+    <t>le soldat</t>
+  </si>
+  <si>
+    <t>la lumière</t>
+  </si>
+  <si>
+    <t>le repas</t>
+  </si>
+  <si>
+    <t>la statue</t>
+  </si>
+  <si>
+    <t>le bâtiment</t>
+  </si>
+  <si>
+    <t>le cuisinier</t>
+  </si>
+  <si>
+    <t>le voyageur</t>
+  </si>
+  <si>
+    <t>le chat</t>
+  </si>
+  <si>
+    <t>la blague</t>
+  </si>
+  <si>
+    <t>le portrait</t>
+  </si>
+  <si>
+    <t>le chercheur</t>
+  </si>
+  <si>
+    <t>le train</t>
+  </si>
+  <si>
+    <t>la cuisine</t>
+  </si>
+  <si>
+    <t>le sac</t>
+  </si>
+  <si>
+    <t>l'athlète</t>
+  </si>
+  <si>
+    <t>l'actrice</t>
+  </si>
+  <si>
+    <t>l'homme</t>
+  </si>
+  <si>
+    <t>l'histoire</t>
+  </si>
+  <si>
+    <t>le bébé</t>
+  </si>
+  <si>
+    <t>le chien</t>
+  </si>
+  <si>
+    <t>le magasin</t>
+  </si>
+  <si>
+    <t>le cheval</t>
+  </si>
+  <si>
+    <t>le thé</t>
+  </si>
+  <si>
+    <t>le garçon</t>
+  </si>
+  <si>
+    <t>la peinture</t>
+  </si>
+  <si>
+    <t>le modèle</t>
+  </si>
+  <si>
+    <t>l'enfant</t>
+  </si>
+  <si>
+    <t>le criminel</t>
+  </si>
+  <si>
+    <t>l'ours</t>
+  </si>
+  <si>
+    <t>le professeur</t>
+  </si>
+  <si>
+    <t>la robe</t>
+  </si>
+  <si>
+    <t>la couverture</t>
+  </si>
+  <si>
+    <t>l'étudiant</t>
+  </si>
+  <si>
+    <t>le propriétaire</t>
+  </si>
+  <si>
+    <t>le candidat</t>
+  </si>
+  <si>
+    <t>scale_first</t>
+  </si>
+  <si>
+    <t>scale_second</t>
+  </si>
+  <si>
+    <t>unique</t>
+  </si>
+  <si>
+    <t>vide</t>
+  </si>
+  <si>
+    <t>insoluble</t>
+  </si>
+  <si>
+    <t>inoubliable</t>
+  </si>
+  <si>
+    <t>inaudible</t>
+  </si>
+  <si>
+    <t>trempé</t>
+  </si>
+  <si>
+    <t>abattu</t>
+  </si>
+  <si>
+    <t>impossible</t>
+  </si>
+  <si>
+    <t>parfait</t>
+  </si>
+  <si>
+    <t>honorable</t>
+  </si>
+  <si>
+    <t>éblouissant</t>
+  </si>
+  <si>
+    <t>épuisé</t>
+  </si>
+  <si>
+    <t>délicieux</t>
+  </si>
+  <si>
+    <t>ancien</t>
+  </si>
+  <si>
+    <t>énorme</t>
+  </si>
+  <si>
+    <t>obèse</t>
+  </si>
+  <si>
+    <t>affamé</t>
+  </si>
+  <si>
+    <t>sublime</t>
+  </si>
+  <si>
+    <t>beau</t>
+  </si>
+  <si>
+    <t>hilarant</t>
+  </si>
+  <si>
+    <t>hideux</t>
+  </si>
+  <si>
+    <t>brilliant</t>
+  </si>
+  <si>
+    <t>rapide</t>
+  </si>
+  <si>
+    <t>propre</t>
+  </si>
+  <si>
+    <t>riche</t>
+  </si>
+  <si>
+    <t>profond</t>
+  </si>
+  <si>
+    <t>lourd</t>
+  </si>
+  <si>
+    <t>grand</t>
+  </si>
+  <si>
+    <t>méchant</t>
+  </si>
+  <si>
+    <t>ouvert</t>
+  </si>
+  <si>
+    <t>blanc</t>
+  </si>
+  <si>
+    <t>chaud</t>
+  </si>
+  <si>
+    <t>paresseux</t>
+  </si>
+  <si>
+    <t>colorée</t>
+  </si>
+  <si>
+    <t>fort</t>
+  </si>
+  <si>
+    <t>curieux</t>
+  </si>
+  <si>
+    <t>dangereux</t>
+  </si>
+  <si>
+    <t>marron</t>
+  </si>
+  <si>
+    <t>raisonnable</t>
+  </si>
+  <si>
+    <t>ennuyeuse</t>
+  </si>
+  <si>
+    <t>fin</t>
+  </si>
+  <si>
+    <t>sérieux</t>
+  </si>
+  <si>
+    <t>pressé</t>
+  </si>
+  <si>
+    <t>inquiet</t>
+  </si>
+  <si>
+    <t>spéciale</t>
+  </si>
+  <si>
+    <t>faible</t>
+  </si>
+  <si>
+    <t>dure</t>
+  </si>
+  <si>
+    <t>mémorable</t>
+  </si>
+  <si>
+    <t>calme</t>
+  </si>
+  <si>
+    <t>mouillé</t>
+  </si>
+  <si>
+    <t>triste</t>
+  </si>
+  <si>
+    <t>difficile</t>
+  </si>
+  <si>
+    <t>bon</t>
+  </si>
+  <si>
+    <t>respectable</t>
+  </si>
+  <si>
+    <t>vif</t>
+  </si>
+  <si>
+    <t>fatigué</t>
+  </si>
+  <si>
+    <t>goûteux</t>
+  </si>
+  <si>
+    <t>vieux</t>
+  </si>
+  <si>
+    <t>gros</t>
+  </si>
+  <si>
+    <t>gras</t>
+  </si>
+  <si>
+    <t>mignon</t>
+  </si>
+  <si>
+    <t>drôle</t>
+  </si>
+  <si>
+    <t>moche</t>
+  </si>
+  <si>
+    <t>intelligent</t>
+  </si>
+  <si>
+    <t>lent</t>
+  </si>
+  <si>
+    <t>sale</t>
+  </si>
+  <si>
+    <t>pauvre</t>
+  </si>
+  <si>
+    <t>superficiel</t>
+  </si>
+  <si>
+    <t>léger</t>
+  </si>
+  <si>
+    <t>petit</t>
+  </si>
+  <si>
+    <t>gentil</t>
+  </si>
+  <si>
+    <t>fermé</t>
+  </si>
+  <si>
+    <t>noir</t>
+  </si>
+  <si>
+    <t>froid</t>
+  </si>
+  <si>
+    <t>actif</t>
+  </si>
+  <si>
+    <t>large</t>
+  </si>
+  <si>
+    <t>joli</t>
+  </si>
+  <si>
+    <t>timide</t>
+  </si>
+  <si>
+    <t>fou</t>
+  </si>
+  <si>
+    <t>effrayant</t>
+  </si>
+  <si>
+    <t>fâché</t>
+  </si>
+  <si>
+    <t>cher</t>
+  </si>
+  <si>
+    <t>doux</t>
+  </si>
+  <si>
+    <t>jeune</t>
+  </si>
+  <si>
+    <t>poli</t>
+  </si>
+  <si>
+    <t>stupide</t>
+  </si>
+  <si>
+    <t>verb</t>
+  </si>
+  <si>
+    <t>est</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>faim</t>
   </si>
 </sst>
 </file>
@@ -508,7 +649,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -786,20 +927,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G45"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="20.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.08984375" customWidth="1"/>
-    <col min="6" max="6" width="28.453125" customWidth="1"/>
-    <col min="7" max="7" width="30.36328125" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
         <v>26</v>
@@ -811,16 +953,22 @@
         <v>0</v>
       </c>
       <c r="E1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F1" t="s">
-        <v>28</v>
+        <v>101</v>
       </c>
       <c r="G1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+        <v>102</v>
+      </c>
+      <c r="H1" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -834,16 +982,22 @@
         <v>27</v>
       </c>
       <c r="E2" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="G2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+        <v>103</v>
+      </c>
+      <c r="H2" t="s">
+        <v>57</v>
+      </c>
+      <c r="I2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -857,16 +1011,22 @@
         <v>27</v>
       </c>
       <c r="E3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>71</v>
+        <v>148</v>
       </c>
       <c r="G3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+        <v>104</v>
+      </c>
+      <c r="H3" t="s">
+        <v>58</v>
+      </c>
+      <c r="I3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -880,16 +1040,22 @@
         <v>27</v>
       </c>
       <c r="E4" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>73</v>
+        <v>149</v>
       </c>
       <c r="G4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+        <v>105</v>
+      </c>
+      <c r="H4" t="s">
+        <v>59</v>
+      </c>
+      <c r="I4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -903,16 +1069,22 @@
         <v>27</v>
       </c>
       <c r="E5" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
-        <v>75</v>
+        <v>150</v>
       </c>
       <c r="G5" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+        <v>106</v>
+      </c>
+      <c r="H5" t="s">
+        <v>60</v>
+      </c>
+      <c r="I5" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -926,16 +1098,22 @@
         <v>27</v>
       </c>
       <c r="E6" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s">
-        <v>79</v>
+        <v>151</v>
       </c>
       <c r="G6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+        <v>107</v>
+      </c>
+      <c r="H6" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -949,16 +1127,22 @@
         <v>27</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>81</v>
+        <v>152</v>
       </c>
       <c r="G7" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+        <v>108</v>
+      </c>
+      <c r="H7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -972,16 +1156,22 @@
         <v>27</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F8" t="s">
-        <v>83</v>
+        <v>153</v>
       </c>
       <c r="G8" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>109</v>
+      </c>
+      <c r="H8" t="s">
+        <v>63</v>
+      </c>
+      <c r="I8" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -995,16 +1185,22 @@
         <v>27</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F9" t="s">
-        <v>85</v>
+        <v>154</v>
       </c>
       <c r="G9" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+        <v>110</v>
+      </c>
+      <c r="H9" t="s">
+        <v>64</v>
+      </c>
+      <c r="I9" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1018,16 +1214,22 @@
         <v>27</v>
       </c>
       <c r="E10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F10" t="s">
-        <v>87</v>
+        <v>155</v>
       </c>
       <c r="G10" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+      <c r="H10" t="s">
+        <v>65</v>
+      </c>
+      <c r="I10" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1041,16 +1243,22 @@
         <v>27</v>
       </c>
       <c r="E11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F11" t="s">
-        <v>89</v>
+        <v>156</v>
       </c>
       <c r="G11" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+        <v>112</v>
+      </c>
+      <c r="H11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I11" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1064,16 +1272,22 @@
         <v>27</v>
       </c>
       <c r="E12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F12" t="s">
-        <v>91</v>
+        <v>157</v>
       </c>
       <c r="G12" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+        <v>113</v>
+      </c>
+      <c r="H12" t="s">
+        <v>67</v>
+      </c>
+      <c r="I12" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1087,16 +1301,22 @@
         <v>27</v>
       </c>
       <c r="E13" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F13" t="s">
-        <v>77</v>
+        <v>158</v>
       </c>
       <c r="G13" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+        <v>114</v>
+      </c>
+      <c r="H13" t="s">
+        <v>80</v>
+      </c>
+      <c r="I13" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1110,16 +1330,22 @@
         <v>27</v>
       </c>
       <c r="E14" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F14" t="s">
-        <v>93</v>
+        <v>159</v>
       </c>
       <c r="G14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+        <v>115</v>
+      </c>
+      <c r="H14" t="s">
+        <v>68</v>
+      </c>
+      <c r="I14" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1133,16 +1359,22 @@
         <v>27</v>
       </c>
       <c r="E15" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F15" t="s">
-        <v>95</v>
+        <v>160</v>
       </c>
       <c r="G15" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+        <v>116</v>
+      </c>
+      <c r="H15" t="s">
+        <v>69</v>
+      </c>
+      <c r="I15" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1156,16 +1388,22 @@
         <v>27</v>
       </c>
       <c r="E16" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F16" t="s">
-        <v>97</v>
+        <v>161</v>
       </c>
       <c r="G16" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+      <c r="H16" t="s">
+        <v>70</v>
+      </c>
+      <c r="I16" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1179,16 +1417,22 @@
         <v>27</v>
       </c>
       <c r="E17" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F17" t="s">
-        <v>99</v>
+        <v>162</v>
       </c>
       <c r="G17" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+        <v>118</v>
+      </c>
+      <c r="H17" t="s">
+        <v>71</v>
+      </c>
+      <c r="I17" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1202,16 +1446,22 @@
         <v>27</v>
       </c>
       <c r="E18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F18" t="s">
-        <v>101</v>
+        <v>192</v>
       </c>
       <c r="G18" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+        <v>119</v>
+      </c>
+      <c r="H18" t="s">
+        <v>72</v>
+      </c>
+      <c r="I18" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1225,16 +1475,22 @@
         <v>27</v>
       </c>
       <c r="E19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F19" t="s">
-        <v>38</v>
+        <v>121</v>
       </c>
       <c r="G19" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+        <v>120</v>
+      </c>
+      <c r="H19" t="s">
+        <v>81</v>
+      </c>
+      <c r="I19" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1248,16 +1504,22 @@
         <v>27</v>
       </c>
       <c r="E20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F20" t="s">
-        <v>105</v>
+        <v>163</v>
       </c>
       <c r="G20" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+        <v>121</v>
+      </c>
+      <c r="H20" t="s">
+        <v>73</v>
+      </c>
+      <c r="I20" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1271,16 +1533,22 @@
         <v>27</v>
       </c>
       <c r="E21" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F21" t="s">
-        <v>107</v>
+        <v>164</v>
       </c>
       <c r="G21" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+        <v>122</v>
+      </c>
+      <c r="H21" t="s">
+        <v>74</v>
+      </c>
+      <c r="I21" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1294,16 +1562,22 @@
         <v>27</v>
       </c>
       <c r="E22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F22" t="s">
-        <v>109</v>
+        <v>165</v>
       </c>
       <c r="G22" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+        <v>123</v>
+      </c>
+      <c r="H22" t="s">
+        <v>75</v>
+      </c>
+      <c r="I22" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1317,457 +1591,596 @@
         <v>27</v>
       </c>
       <c r="E23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F23" t="s">
-        <v>110</v>
+        <v>166</v>
       </c>
       <c r="G23" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+      <c r="H23" t="s">
+        <v>76</v>
+      </c>
+      <c r="I23" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E24" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F24" t="s">
-        <v>37</v>
+        <v>167</v>
       </c>
       <c r="G24" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+        <v>125</v>
+      </c>
+      <c r="H24" t="s">
+        <v>77</v>
+      </c>
+      <c r="I24" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="D25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E25" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F25" t="s">
-        <v>52</v>
+        <v>168</v>
       </c>
       <c r="G25" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+      <c r="H25" t="s">
+        <v>78</v>
+      </c>
+      <c r="I25" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="D26" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E26" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F26" t="s">
-        <v>54</v>
+        <v>169</v>
       </c>
       <c r="G26" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+        <v>127</v>
+      </c>
+      <c r="H26" t="s">
+        <v>82</v>
+      </c>
+      <c r="I26" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D27" t="s">
+        <v>29</v>
+      </c>
+      <c r="E27" t="s">
+        <v>34</v>
+      </c>
+      <c r="F27" t="s">
+        <v>170</v>
+      </c>
+      <c r="G27" t="s">
+        <v>128</v>
+      </c>
+      <c r="H27" t="s">
+        <v>83</v>
+      </c>
+      <c r="I27" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D27" t="s">
-        <v>30</v>
-      </c>
-      <c r="E27" t="s">
-        <v>40</v>
-      </c>
-      <c r="F27" t="s">
-        <v>56</v>
-      </c>
-      <c r="G27" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>113</v>
-      </c>
       <c r="D28" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E28" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F28" t="s">
-        <v>114</v>
+        <v>171</v>
       </c>
       <c r="G28" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+        <v>129</v>
+      </c>
+      <c r="H28" t="s">
+        <v>79</v>
+      </c>
+      <c r="I28" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D29" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E29" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F29" t="s">
-        <v>58</v>
+        <v>172</v>
       </c>
       <c r="G29" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+        <v>130</v>
+      </c>
+      <c r="H29" t="s">
+        <v>84</v>
+      </c>
+      <c r="I29" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="D30" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E30" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F30" t="s">
-        <v>60</v>
+        <v>173</v>
       </c>
       <c r="G30" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+        <v>131</v>
+      </c>
+      <c r="H30" t="s">
+        <v>85</v>
+      </c>
+      <c r="I30" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="D31" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E31" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F31" t="s">
-        <v>62</v>
+        <v>174</v>
       </c>
       <c r="G31" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+      <c r="H31" t="s">
+        <v>86</v>
+      </c>
+      <c r="I31" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="D32" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F32" t="s">
-        <v>103</v>
+        <v>175</v>
       </c>
       <c r="G32" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+        <v>133</v>
+      </c>
+      <c r="H32" t="s">
+        <v>87</v>
+      </c>
+      <c r="I32" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="D33" t="s">
+        <v>29</v>
+      </c>
+      <c r="E33" t="s">
+        <v>33</v>
+      </c>
+      <c r="F33" t="s">
+        <v>176</v>
+      </c>
+      <c r="G33" t="s">
+        <v>134</v>
+      </c>
+      <c r="H33" t="s">
+        <v>88</v>
+      </c>
+      <c r="I33" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D34" t="s">
+        <v>29</v>
+      </c>
+      <c r="E34" t="s">
+        <v>33</v>
+      </c>
+      <c r="F34" t="s">
+        <v>177</v>
+      </c>
+      <c r="G34" t="s">
+        <v>135</v>
+      </c>
+      <c r="H34" t="s">
+        <v>89</v>
+      </c>
+      <c r="I34" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D35" t="s">
         <v>30</v>
       </c>
-      <c r="E33" t="s">
-        <v>34</v>
-      </c>
-      <c r="F33" t="s">
-        <v>67</v>
-      </c>
-      <c r="G33" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34">
-        <v>33</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D34" t="s">
-        <v>30</v>
-      </c>
-      <c r="E34" t="s">
-        <v>34</v>
-      </c>
-      <c r="F34" t="s">
-        <v>64</v>
-      </c>
-      <c r="G34" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35">
-        <v>34</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D35" t="s">
-        <v>31</v>
-      </c>
       <c r="E35" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F35" t="s">
-        <v>41</v>
+        <v>178</v>
       </c>
       <c r="G35" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+        <v>136</v>
+      </c>
+      <c r="H35" t="s">
+        <v>90</v>
+      </c>
+      <c r="I35" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>117</v>
+        <v>46</v>
       </c>
       <c r="D36" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E36" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F36" t="s">
-        <v>116</v>
+        <v>179</v>
       </c>
       <c r="G36" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+        <v>137</v>
+      </c>
+      <c r="H36" t="s">
+        <v>91</v>
+      </c>
+      <c r="I36" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>120</v>
+        <v>47</v>
       </c>
       <c r="D37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E37" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F37" t="s">
-        <v>119</v>
+        <v>180</v>
       </c>
       <c r="G37" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+        <v>138</v>
+      </c>
+      <c r="H37" t="s">
+        <v>92</v>
+      </c>
+      <c r="I37" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>122</v>
+        <v>48</v>
       </c>
       <c r="D38" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E38" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F38" t="s">
-        <v>123</v>
+        <v>181</v>
       </c>
       <c r="G38" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+        <v>139</v>
+      </c>
+      <c r="H38" t="s">
+        <v>93</v>
+      </c>
+      <c r="I38" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>126</v>
+        <v>49</v>
       </c>
       <c r="D39" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E39" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F39" t="s">
-        <v>125</v>
+        <v>182</v>
       </c>
       <c r="G39" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+        <v>140</v>
+      </c>
+      <c r="H39" t="s">
+        <v>94</v>
+      </c>
+      <c r="I39" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>129</v>
+        <v>50</v>
       </c>
       <c r="D40" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E40" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F40" t="s">
-        <v>128</v>
+        <v>183</v>
       </c>
       <c r="G40" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+      <c r="H40" t="s">
+        <v>95</v>
+      </c>
+      <c r="I40" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>132</v>
+        <v>51</v>
       </c>
       <c r="D41" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E41" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F41" t="s">
-        <v>131</v>
+        <v>184</v>
       </c>
       <c r="G41" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+        <v>142</v>
+      </c>
+      <c r="H41" t="s">
+        <v>96</v>
+      </c>
+      <c r="I41" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>136</v>
+        <v>52</v>
       </c>
       <c r="D42" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E42" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F42" t="s">
-        <v>134</v>
+        <v>185</v>
       </c>
       <c r="G42" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+        <v>143</v>
+      </c>
+      <c r="H42" t="s">
+        <v>97</v>
+      </c>
+      <c r="I42" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>138</v>
+        <v>53</v>
       </c>
       <c r="D43" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E43" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F43" t="s">
-        <v>137</v>
+        <v>186</v>
       </c>
       <c r="G43" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+        <v>144</v>
+      </c>
+      <c r="H43" t="s">
+        <v>98</v>
+      </c>
+      <c r="I43" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>142</v>
+        <v>54</v>
       </c>
       <c r="D44" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E44" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F44" t="s">
-        <v>140</v>
+        <v>187</v>
       </c>
       <c r="G44" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+        <v>145</v>
+      </c>
+      <c r="H44" t="s">
+        <v>99</v>
+      </c>
+      <c r="I44" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>145</v>
+        <v>55</v>
       </c>
       <c r="D45" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E45" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F45" t="s">
-        <v>143</v>
+        <v>188</v>
       </c>
       <c r="G45" t="s">
-        <v>144</v>
+        <v>146</v>
+      </c>
+      <c r="H45" t="s">
+        <v>100</v>
+      </c>
+      <c r="I45" t="s">
+        <v>190</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G45" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H45" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>